<commit_message>
Update change to Staffing Tools
</commit_message>
<xml_diff>
--- a/temp_update.xlsx
+++ b/temp_update.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cb4a1c0c7a4389a8/Documents/GitHub/GoLive_Staffing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6D1E8AB-277B-4132-A7AB-E431F6A688F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{A6D1E8AB-277B-4132-A7AB-E431F6A688F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C8D15E9E-BD45-4D34-A4B0-67BECB5FAE8E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">report!$A$1:$I$1018</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>

</xml_diff>